<commit_message>
refactor: Revise expedition effect handling and update data structures
- Replaced the previous ExpeditionEventEffectConfig with a more flexible ExpeditionEffectConfig structure to accommodate various effect types.
- Updated combat encounter and event option configurations to utilize lists of effects for victory and defeat scenarios.
- Refactored gameplay logic to handle new effect configurations, enhancing clarity and maintainability.
- Adjusted UI components to reflect changes in money management instead of crystal rewards, improving user experience.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition_combat_encounter.xlsx
+++ b/Configs/GameConfig/Datas/expedition_combat_encounter.xlsx
@@ -43,10 +43,10 @@
     <t>description</t>
   </si>
   <si>
-    <t>victory_crystal_reward</t>
-  </si>
-  <si>
-    <t>victory_exp_reward</t>
+    <t>*lst_victory_effect</t>
+  </si>
+  <si>
+    <t>*lst_defeat_effect</t>
   </si>
   <si>
     <t>*enemy_marbles</t>
@@ -76,10 +76,10 @@
     <t>敌方巡逻 Marble 正在封锁出口，击败它们即可带走补给。</t>
   </si>
   <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>15</t>
+    <t>add_money,获得120晶体,120</t>
+  </si>
+  <si>
+    <t>add_player_marble_exp,全队获得 15 经验, 15</t>
   </si>
   <si>
     <t>soldier</t>
@@ -1170,7 +1170,8 @@
     <col min="2" max="2" width="23.8181818181818" style="5" customWidth="1"/>
     <col min="3" max="3" width="12.2727272727273" style="5" customWidth="1"/>
     <col min="4" max="4" width="61.7272727272727" style="5" customWidth="1"/>
-    <col min="5" max="6" width="27.5454545454545" style="5" customWidth="1"/>
+    <col min="5" max="5" width="33.2727272727273" style="5" customWidth="1"/>
+    <col min="6" max="6" width="53.9090909090909" style="5" customWidth="1"/>
     <col min="7" max="7" width="10.3636363636364" style="5" customWidth="1"/>
     <col min="8" max="8" width="11.5454545454545" style="5" customWidth="1"/>
     <col min="9" max="9" width="15.2727272727273" style="5" customWidth="1"/>
@@ -1193,7 +1194,7 @@
       <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="9" t="s">

</xml_diff>

<commit_message>
refactor: Integrate camp and initial configurations into expedition flow
- Introduced new configuration files for camp and initial states, allowing for dynamic setup of player starting conditions.
- Updated existing expedition configurations to utilize the new MarbleSpawnConfig for enemy marbles, enhancing consistency across gameplay elements.
- Refactored gameplay logic to support the new camp and initial configurations, ensuring proper initialization of player resources and marble setups.
- Renamed combat-related identifiers to CombatSide to clarify the distinction between configuration and runtime enemy relationships.
- Streamlined data handling in the ExpeditionCombatSessionController and related classes to accommodate the new configuration structure.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition_combat_encounter.xlsx
+++ b/Configs/GameConfig/Datas/expedition_combat_encounter.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
   <si>
     <t>##var</t>
   </si>
@@ -52,18 +52,15 @@
     <t>*enemy_marbles</t>
   </si>
   <si>
-    <t>enemy_config_id</t>
-  </si>
-  <si>
     <t>marble_config_id</t>
   </si>
   <si>
-    <t>display_name</t>
-  </si>
-  <si>
     <t>level</t>
   </si>
   <si>
+    <t>camp_config_id</t>
+  </si>
+  <si>
     <t>##type</t>
   </si>
   <si>
@@ -91,13 +88,10 @@
     <t>soldier</t>
   </si>
   <si>
-    <t>巡逻剑士</t>
+    <t>human</t>
   </si>
   <si>
     <t>archer</t>
-  </si>
-  <si>
-    <t>巡逻弓箭手</t>
   </si>
 </sst>
 </file>
@@ -495,6 +489,19 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -522,19 +529,6 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -791,7 +785,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -810,23 +804,29 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -834,16 +834,25 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1171,240 +1180,223 @@
     <col min="6" max="6" width="53.9090909090909" style="5" customWidth="1"/>
     <col min="7" max="7" width="18.9090909090909" style="5" customWidth="1"/>
     <col min="8" max="8" width="20.1818181818182" style="5" customWidth="1"/>
-    <col min="9" max="9" width="15.2727272727273" style="5" customWidth="1"/>
-    <col min="10" max="17" width="9" style="5"/>
+    <col min="9" max="9" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="10" max="10" width="9" style="6"/>
+    <col min="11" max="17" width="9" style="5"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:17">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:17">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:17">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" s="2" customFormat="1" spans="1:17">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="C4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
+      <c r="I4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="16"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
     </row>
     <row r="5" s="3" customFormat="1" spans="1:17">
-      <c r="A5" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
+      <c r="A5" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
     </row>
     <row r="6" s="3" customFormat="1" spans="1:17">
-      <c r="A6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
+      <c r="A6" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
     </row>
     <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:17">
-      <c r="A7" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="16"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="17"/>
+      <c r="A7" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="20"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="21"/>
     </row>
     <row r="8" spans="1:17">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18" t="s">
+      <c r="A8" s="23"/>
+      <c r="B8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="G8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="5">
-        <v>1</v>
-      </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="5">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="5">
-        <v>0</v>
-      </c>
+      <c r="P8"/>
+      <c r="Q8"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="G9" s="5">
-        <v>2</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>21</v>
+      <c r="A9" s="23"/>
+      <c r="B9" s="23"/>
+      <c r="G9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="5">
-        <v>0</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="P9"/>
+      <c r="Q9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="G1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
refactor: Transition to tier-based reward system and update expedition configurations
- Replaced the EnumExpeditionRewardOperation with a tier-based system for reward operations in expedition effects.
- Updated AddMoneyEffect, AddPlayerMarbleExpEffect, and AddPlayerMarbleHpEffect to utilize the new tier and value parameters for dynamic reward calculations.
- Removed deprecated ExpeditionScaledValueConfig and EnumExpeditionRewardOperation classes to streamline the codebase.
- Adjusted related XML and JSON configuration files to align with the new reward structure, enhancing clarity and maintainability.
- Improved documentation and comments throughout the code to reflect the changes in the expedition reward handling.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition_combat_encounter.xlsx
+++ b/Configs/GameConfig/Datas/expedition_combat_encounter.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="37">
   <si>
     <t>##var</t>
   </si>
@@ -55,6 +55,33 @@
     <t>*enemy_marbles</t>
   </si>
   <si>
+    <t>$type</t>
+  </si>
+  <si>
+    <t>operation</t>
+  </si>
+  <si>
+    <t>tier</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>marble_count_tier</t>
+  </si>
+  <si>
+    <t>marble_count_value</t>
+  </si>
+  <si>
+    <t>marble_type_tier</t>
+  </si>
+  <si>
+    <t>marble_type_value</t>
+  </si>
+  <si>
+    <t>summary</t>
+  </si>
+  <si>
     <t>marble_config_id</t>
   </si>
   <si>
@@ -70,9 +97,18 @@
     <t>string</t>
   </si>
   <si>
+    <t>EnumOperation</t>
+  </si>
+  <si>
+    <t>EnumExpeditionRewardTier</t>
+  </si>
+  <si>
     <t>int</t>
   </si>
   <si>
+    <t>MarbleSpawnConfig</t>
+  </si>
+  <si>
     <t>##</t>
   </si>
   <si>
@@ -82,10 +118,19 @@
     <t>敌方巡逻 Marble 正在封锁出口，击败它们即可带走补给。</t>
   </si>
   <si>
-    <t>add_money,获得{money}晶体,add,large</t>
-  </si>
-  <si>
-    <t>add_player_marble_exp,全队获得 {exp} 经验, tiny</t>
+    <t>add_money</t>
+  </si>
+  <si>
+    <t>add</t>
+  </si>
+  <si>
+    <t>large</t>
+  </si>
+  <si>
+    <t>获得{money}晶体</t>
+  </si>
+  <si>
+    <t>tiny</t>
   </si>
   <si>
     <t>soldier</t>
@@ -480,7 +525,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -504,7 +549,22 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -518,6 +578,34 @@
     </border>
     <border>
       <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color auto="1"/>
       </left>
       <right/>
@@ -538,6 +626,37 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -664,7 +783,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
@@ -676,34 +795,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="10">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="14">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="15">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="16">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="0">
@@ -788,7 +907,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -810,25 +929,58 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -840,6 +992,15 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -849,6 +1010,15 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -858,7 +1028,28 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1172,245 +1363,464 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:AH9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5"/>
     <col min="2" max="2" width="32.4545454545455" style="5" customWidth="1"/>
     <col min="3" max="3" width="12.2727272727273" style="5" customWidth="1"/>
-    <col min="4" max="4" width="61.7272727272727" style="5" customWidth="1"/>
-    <col min="5" max="5" width="43.0909090909091" style="5" customWidth="1"/>
-    <col min="6" max="6" width="53.9090909090909" style="5" customWidth="1"/>
-    <col min="7" max="7" width="26.2727272727273" style="5" customWidth="1"/>
-    <col min="8" max="8" width="18.9090909090909" style="5" customWidth="1"/>
-    <col min="9" max="9" width="20.1818181818182" style="5" customWidth="1"/>
-    <col min="10" max="10" width="17.7272727272727" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9" style="6"/>
-    <col min="12" max="18" width="9" style="5"/>
+    <col min="4" max="4" width="61.7272727272727" style="6" customWidth="1"/>
+    <col min="5" max="5" width="11.5454545454545" style="7" customWidth="1"/>
+    <col min="6" max="6" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="7" max="7" width="8" style="5" customWidth="1"/>
+    <col min="8" max="8" width="7.45454545454545" style="5" customWidth="1"/>
+    <col min="9" max="9" width="10.6363636363636" style="5" customWidth="1"/>
+    <col min="10" max="10" width="10.5454545454545" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9.90909090909091" style="5" customWidth="1"/>
+    <col min="12" max="12" width="8.72727272727273" style="5" customWidth="1"/>
+    <col min="13" max="13" width="18.5454545454545" style="8" customWidth="1"/>
+    <col min="14" max="14" width="11.5454545454545" style="7" customWidth="1"/>
+    <col min="15" max="15" width="16.4545454545455" style="5" customWidth="1"/>
+    <col min="16" max="16" width="8" style="5" customWidth="1"/>
+    <col min="17" max="17" width="7.45454545454545" style="5" customWidth="1"/>
+    <col min="18" max="18" width="10.6363636363636" style="5" customWidth="1"/>
+    <col min="19" max="19" width="10.5454545454545" style="5" customWidth="1"/>
+    <col min="20" max="20" width="9.90909090909091" style="5" customWidth="1"/>
+    <col min="21" max="21" width="8.72727272727273" style="5" customWidth="1"/>
+    <col min="22" max="22" width="18.5454545454545" style="8" customWidth="1"/>
+    <col min="23" max="23" width="26.2727272727273" style="9" customWidth="1"/>
+    <col min="24" max="24" width="18.9090909090909" style="5" customWidth="1"/>
+    <col min="25" max="25" width="20.1818181818182" style="5" customWidth="1"/>
+    <col min="26" max="26" width="17.7272727272727" style="5" customWidth="1"/>
+    <col min="27" max="27" width="9" style="9"/>
+    <col min="28" max="34" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:18">
-      <c r="A1" s="7" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:34">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="15"/>
+      <c r="W1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="X1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
+      <c r="Y1" s="18"/>
+      <c r="Z1" s="19"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="11"/>
+      <c r="AD1" s="11"/>
+      <c r="AE1" s="11"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="11"/>
+      <c r="AH1" s="11"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:18">
-      <c r="A2" s="7" t="s">
+    <row r="2" s="1" customFormat="1" spans="1:34">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="F2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="G2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
+      <c r="H2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="M2" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="U2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="V2" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="W2" s="20"/>
+      <c r="X2" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y2" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z2" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA2" s="20"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:18">
-      <c r="A3" s="7" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:34">
+      <c r="A3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="23"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
+      <c r="AA3" s="20"/>
+      <c r="AB3" s="11"/>
+      <c r="AC3" s="11"/>
+      <c r="AD3" s="11"/>
+      <c r="AE3" s="11"/>
+      <c r="AF3" s="11"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:18">
-      <c r="A4" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="K4" s="16"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
+    <row r="4" s="2" customFormat="1" spans="1:34">
+      <c r="A4" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="28"/>
+      <c r="F4" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="N4" s="28"/>
+      <c r="O4" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="S4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="T4" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="U4" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="W4" s="30"/>
+      <c r="X4" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y4" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z4" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA4" s="30"/>
+      <c r="AB4" s="26"/>
+      <c r="AC4" s="26"/>
+      <c r="AD4" s="26"/>
+      <c r="AE4" s="26"/>
+      <c r="AF4" s="26"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:18">
-      <c r="A5" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
+    <row r="5" s="3" customFormat="1" spans="1:34">
+      <c r="A5" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="31"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="35"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="32"/>
+      <c r="R5" s="32"/>
+      <c r="S5" s="32"/>
+      <c r="T5" s="32"/>
+      <c r="U5" s="32"/>
+      <c r="V5" s="35"/>
+      <c r="W5" s="36"/>
+      <c r="X5" s="32"/>
+      <c r="Y5" s="32"/>
+      <c r="Z5" s="32"/>
+      <c r="AA5" s="36"/>
+      <c r="AB5" s="32"/>
+      <c r="AC5" s="32"/>
+      <c r="AD5" s="32"/>
+      <c r="AE5" s="32"/>
+      <c r="AF5" s="32"/>
     </row>
-    <row r="6" s="3" customFormat="1" spans="1:18">
-      <c r="A6" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
+    <row r="6" s="3" customFormat="1" spans="1:34">
+      <c r="A6" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="31"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32"/>
+      <c r="R6" s="32"/>
+      <c r="S6" s="32"/>
+      <c r="T6" s="32"/>
+      <c r="U6" s="32"/>
+      <c r="V6" s="35"/>
+      <c r="W6" s="36"/>
+      <c r="X6" s="32"/>
+      <c r="Y6" s="32"/>
+      <c r="Z6" s="32"/>
+      <c r="AA6" s="36"/>
+      <c r="AB6" s="32"/>
+      <c r="AC6" s="32"/>
+      <c r="AD6" s="32"/>
+      <c r="AE6" s="32"/>
+      <c r="AF6" s="32"/>
     </row>
-    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:18">
-      <c r="A7" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
+    <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:34">
+      <c r="A7" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="37"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="38"/>
+      <c r="I7" s="38"/>
+      <c r="J7" s="38"/>
+      <c r="K7" s="38"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="40"/>
+      <c r="O7" s="38"/>
+      <c r="P7" s="38"/>
+      <c r="Q7" s="38"/>
+      <c r="R7" s="38"/>
+      <c r="S7" s="38"/>
+      <c r="T7" s="38"/>
+      <c r="U7" s="38"/>
+      <c r="V7" s="41"/>
+      <c r="W7" s="42"/>
+      <c r="X7" s="38"/>
+      <c r="Y7" s="38"/>
+      <c r="Z7" s="38"/>
+      <c r="AA7" s="42"/>
+      <c r="AB7" s="38"/>
+      <c r="AC7" s="38"/>
+      <c r="AD7" s="38"/>
+      <c r="AE7" s="38"/>
+      <c r="AF7" s="38"/>
     </row>
-    <row r="8" spans="1:18">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="23"/>
-      <c r="H8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="I8" s="5">
+    <row r="8" spans="1:34">
+      <c r="A8" s="43"/>
+      <c r="B8" s="43" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="N8" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="O8" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="P8" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="43"/>
+      <c r="R8" s="43"/>
+      <c r="S8" s="43"/>
+      <c r="T8" s="43"/>
+      <c r="U8" s="43"/>
+      <c r="V8" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="W8" s="47"/>
+      <c r="X8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y8" s="5">
         <v>0</v>
       </c>
-      <c r="J8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q8"/>
-      <c r="R8"/>
+      <c r="Z8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG8"/>
+      <c r="AH8"/>
     </row>
-    <row r="9" spans="1:18">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="H9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="5">
+    <row r="9" spans="1:34">
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="X9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y9" s="5">
         <v>0</v>
       </c>
-      <c r="J9" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q9"/>
-      <c r="R9"/>
+      <c r="Z9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG9"/>
+      <c r="AH9"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="H1:J1"/>
+  <mergeCells count="3">
+    <mergeCell ref="E1:M1"/>
+    <mergeCell ref="N1:V1"/>
+    <mergeCell ref="X1:Z1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>